<commit_message>
Add gene-symbol mapping; standardize on "Gene Symbol" column
- mapping.fill_gene_symbols: fill blank gene symbols from the UniProt accession
  (reuses annotations.fetch_annotations); creates the column if absent, leaves
  populated rows untouched, raises AnnotationServiceError if UniProt unreachable
- DEFAULT_GENE_COLUMN = "Gene Symbol"; plots (label_col) and crossdataset
  (label_cols) now default to it, replacing the old "Gene" references
- sample data generator emits a "Gene Symbol" column with a few intentional
  blanks to demonstrate the mapping
- notebook: new step 2b (map gene symbols); all "Gene" references updated to
  "Gene Symbol"
- tests for fill_gene_symbols (offline-safe paths); README updated

https://claude.ai/code/session_01AuJShVNE6C39yUP4goD6fY
</commit_message>
<xml_diff>
--- a/sample_data/sample_dataset.xlsx
+++ b/sample_data/sample_dataset.xlsx
@@ -424,7 +424,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Gene</t>
+          <t>Gene Symbol</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
@@ -756,11 +756,7 @@
           <t>P00003</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>GENE3</t>
-        </is>
-      </c>
+      <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr">
         <is>
           <t>Example protein</t>
@@ -1582,11 +1578,7 @@
           <t>P00017</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>GENE17</t>
-        </is>
-      </c>
+      <c r="B19" t="inlineStr"/>
       <c r="C19" t="inlineStr">
         <is>
           <t>Example protein</t>
@@ -3057,11 +3049,7 @@
           <t>P00042</t>
         </is>
       </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>GENE42</t>
-        </is>
-      </c>
+      <c r="B44" t="inlineStr"/>
       <c r="C44" t="inlineStr">
         <is>
           <t>Example protein</t>

</xml_diff>